<commit_message>
Update Endocrine quarterly counts Excel with TOTAL row and Category table
</commit_message>
<xml_diff>
--- a/dataset/Growth and Endocrine Model/Endocrine_Counts_2021_2025.xlsx
+++ b/dataset/Growth and Endocrine Model/Endocrine_Counts_2021_2025.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,8 +47,19 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +74,48 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00303F9F"/>
+        <bgColor rgb="00303F9F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00008080"/>
+        <bgColor rgb="00008080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E7D32"/>
+        <bgColor rgb="002E7D32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EF6C00"/>
+        <bgColor rgb="00EF6C00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C62828"/>
+        <bgColor rgb="00C62828"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006A1B9A"/>
+        <bgColor rgb="006A1B9A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008D6E63"/>
+        <bgColor rgb="008D6E63"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E3F2FD"/>
         <bgColor rgb="00E3F2FD"/>
       </patternFill>
@@ -115,8 +168,14 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+        <bgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -138,11 +197,25 @@
         <color rgb="00D3D3D3"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00333333"/>
+      </top>
+      <bottom style="double">
+        <color rgb="00333333"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -153,32 +226,72 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -545,18 +658,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
@@ -592,7 +705,7 @@
           <t>Q#</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Total
 Pediatric
@@ -606,37 +719,37 @@
 Patients</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Endocrine
 All Drugs</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Somatropin
 Only</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Levothyroxine
 Only</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>Hydrocortisone
 Only</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>Leuprolide
 Only</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="10" t="inlineStr">
         <is>
           <t>Methimazole
 Only</t>
@@ -644,749 +757,1029 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>2021Q1</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="11" t="n">
         <v>2021</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="12" t="n">
         <v>28359</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="13" t="n">
         <v>291</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="14" t="n">
         <v>855</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="15" t="n">
         <v>400</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="H5" s="16" t="n">
         <v>204</v>
       </c>
-      <c r="I5" s="9" t="n">
+      <c r="I5" s="17" t="n">
         <v>231</v>
       </c>
-      <c r="J5" s="10" t="n">
+      <c r="J5" s="18" t="n">
         <v>43</v>
       </c>
-      <c r="K5" s="11" t="n">
+      <c r="K5" s="19" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>2021Q2</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="20" t="n">
         <v>2021</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="21" t="n">
         <v>29401</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="21" t="n">
         <v>305</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="21" t="n">
         <v>882</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="21" t="n">
         <v>385</v>
       </c>
-      <c r="H6" s="12" t="n">
+      <c r="H6" s="21" t="n">
         <v>256</v>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="21" t="n">
         <v>224</v>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="21" t="n">
         <v>38</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="K6" s="21" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>2021Q3</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="11" t="n">
         <v>2021</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="12" t="n">
         <v>25312</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="13" t="n">
         <v>367</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="14" t="n">
         <v>1180</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G7" s="15" t="n">
         <v>572</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="16" t="n">
         <v>236</v>
       </c>
-      <c r="I7" s="9" t="n">
+      <c r="I7" s="17" t="n">
         <v>262</v>
       </c>
-      <c r="J7" s="10" t="n">
+      <c r="J7" s="18" t="n">
         <v>147</v>
       </c>
-      <c r="K7" s="11" t="n">
+      <c r="K7" s="19" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>2021Q4</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="20" t="n">
         <v>2021</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="21" t="n">
         <v>26855</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="21" t="n">
         <v>532</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="21" t="n">
         <v>1807</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="21" t="n">
         <v>1327</v>
       </c>
-      <c r="H8" s="12" t="n">
+      <c r="H8" s="21" t="n">
         <v>276</v>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="I8" s="21" t="n">
         <v>208</v>
       </c>
-      <c r="J8" s="12" t="n">
+      <c r="J8" s="21" t="n">
         <v>59</v>
       </c>
-      <c r="K8" s="12" t="n">
+      <c r="K8" s="21" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>2022Q1</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="11" t="n">
         <v>2022</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="12" t="n">
         <v>27683</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="13" t="n">
         <v>543</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="14" t="n">
         <v>1959</v>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="G9" s="15" t="n">
         <v>1405</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="16" t="n">
         <v>331</v>
       </c>
-      <c r="I9" s="9" t="n">
+      <c r="I9" s="17" t="n">
         <v>226</v>
       </c>
-      <c r="J9" s="10" t="n">
+      <c r="J9" s="18" t="n">
         <v>35</v>
       </c>
-      <c r="K9" s="11" t="n">
+      <c r="K9" s="19" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>2022Q2</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="20" t="n">
         <v>2022</v>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="21" t="n">
         <v>25896</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="21" t="n">
         <v>499</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="21" t="n">
         <v>1811</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="21" t="n">
         <v>1197</v>
       </c>
-      <c r="H10" s="12" t="n">
+      <c r="H10" s="21" t="n">
         <v>264</v>
       </c>
-      <c r="I10" s="12" t="n">
+      <c r="I10" s="21" t="n">
         <v>314</v>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="21" t="n">
         <v>65</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="K10" s="21" t="n">
         <v>17</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>2022Q3</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="11" t="n">
         <v>2022</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="12" t="n">
         <v>27166</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="13" t="n">
         <v>434</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="14" t="n">
         <v>1637</v>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="G11" s="15" t="n">
         <v>968</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="16" t="n">
         <v>326</v>
       </c>
-      <c r="I11" s="9" t="n">
+      <c r="I11" s="17" t="n">
         <v>291</v>
       </c>
-      <c r="J11" s="10" t="n">
+      <c r="J11" s="18" t="n">
         <v>91</v>
       </c>
-      <c r="K11" s="11" t="n">
+      <c r="K11" s="19" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>2022Q4</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="20" t="n">
         <v>2022</v>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="21" t="n">
         <v>29025</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="21" t="n">
         <v>586</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="21" t="n">
         <v>1854</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="21" t="n">
         <v>1219</v>
       </c>
-      <c r="H12" s="12" t="n">
+      <c r="H12" s="21" t="n">
         <v>392</v>
       </c>
-      <c r="I12" s="12" t="n">
+      <c r="I12" s="21" t="n">
         <v>248</v>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="21" t="n">
         <v>49</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="K12" s="21" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>2023Q1</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="11" t="n">
         <v>2023</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="12" t="n">
         <v>29901</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="13" t="n">
         <v>568</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="14" t="n">
         <v>1818</v>
       </c>
-      <c r="G13" s="7" t="n">
+      <c r="G13" s="15" t="n">
         <v>1136</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="16" t="n">
         <v>405</v>
       </c>
-      <c r="I13" s="9" t="n">
+      <c r="I13" s="17" t="n">
         <v>231</v>
       </c>
-      <c r="J13" s="10" t="n">
+      <c r="J13" s="18" t="n">
         <v>85</v>
       </c>
-      <c r="K13" s="11" t="n">
+      <c r="K13" s="19" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>2023Q2</t>
         </is>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="20" t="n">
         <v>2023</v>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="21" t="n">
         <v>28603</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="21" t="n">
         <v>581</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="21" t="n">
         <v>2096</v>
       </c>
-      <c r="G14" s="12" t="n">
+      <c r="G14" s="21" t="n">
         <v>1516</v>
       </c>
-      <c r="H14" s="12" t="n">
+      <c r="H14" s="21" t="n">
         <v>335</v>
       </c>
-      <c r="I14" s="12" t="n">
+      <c r="I14" s="21" t="n">
         <v>216</v>
       </c>
-      <c r="J14" s="12" t="n">
+      <c r="J14" s="21" t="n">
         <v>73</v>
       </c>
-      <c r="K14" s="12" t="n">
+      <c r="K14" s="21" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>2023Q3</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="11" t="n">
         <v>2023</v>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="12" t="n">
         <v>28690</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="13" t="n">
         <v>641</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="14" t="n">
         <v>2257</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="G15" s="15" t="n">
         <v>1563</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H15" s="16" t="n">
         <v>365</v>
       </c>
-      <c r="I15" s="9" t="n">
+      <c r="I15" s="17" t="n">
         <v>249</v>
       </c>
-      <c r="J15" s="10" t="n">
+      <c r="J15" s="18" t="n">
         <v>133</v>
       </c>
-      <c r="K15" s="11" t="n">
+      <c r="K15" s="19" t="n">
         <v>17</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>2023Q4</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B16" s="20" t="n">
         <v>2023</v>
       </c>
-      <c r="C16" s="12" t="n">
+      <c r="C16" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D16" s="12" t="n">
+      <c r="D16" s="21" t="n">
         <v>27752</v>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="E16" s="21" t="n">
         <v>754</v>
       </c>
-      <c r="F16" s="12" t="n">
+      <c r="F16" s="21" t="n">
         <v>2682</v>
       </c>
-      <c r="G16" s="12" t="n">
+      <c r="G16" s="21" t="n">
         <v>2097</v>
       </c>
-      <c r="H16" s="12" t="n">
+      <c r="H16" s="21" t="n">
         <v>350</v>
       </c>
-      <c r="I16" s="12" t="n">
+      <c r="I16" s="21" t="n">
         <v>208</v>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="21" t="n">
         <v>90</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="K16" s="21" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>2024Q1</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B17" s="11" t="n">
         <v>2024</v>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="12" t="n">
         <v>29564</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="13" t="n">
         <v>897</v>
       </c>
-      <c r="F17" s="6" t="n">
+      <c r="F17" s="14" t="n">
         <v>3297</v>
       </c>
-      <c r="G17" s="7" t="n">
+      <c r="G17" s="15" t="n">
         <v>2782</v>
       </c>
-      <c r="H17" s="8" t="n">
+      <c r="H17" s="16" t="n">
         <v>306</v>
       </c>
-      <c r="I17" s="9" t="n">
+      <c r="I17" s="17" t="n">
         <v>223</v>
       </c>
-      <c r="J17" s="10" t="n">
+      <c r="J17" s="18" t="n">
         <v>85</v>
       </c>
-      <c r="K17" s="11" t="n">
+      <c r="K17" s="19" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>2024Q2</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n">
+      <c r="B18" s="20" t="n">
         <v>2024</v>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D18" s="21" t="n">
         <v>27944</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="21" t="n">
         <v>813</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F18" s="21" t="n">
         <v>2303</v>
       </c>
-      <c r="G18" s="12" t="n">
+      <c r="G18" s="21" t="n">
         <v>1669</v>
       </c>
-      <c r="H18" s="12" t="n">
+      <c r="H18" s="21" t="n">
         <v>302</v>
       </c>
-      <c r="I18" s="12" t="n">
+      <c r="I18" s="21" t="n">
         <v>250</v>
       </c>
-      <c r="J18" s="12" t="n">
+      <c r="J18" s="21" t="n">
         <v>160</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="K18" s="21" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>2024Q3</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n">
+      <c r="B19" s="11" t="n">
         <v>2024</v>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="D19" s="5" t="n">
+      <c r="D19" s="12" t="n">
         <v>31009</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="13" t="n">
         <v>714</v>
       </c>
-      <c r="F19" s="6" t="n">
+      <c r="F19" s="14" t="n">
         <v>2010</v>
       </c>
-      <c r="G19" s="7" t="n">
+      <c r="G19" s="15" t="n">
         <v>1322</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="H19" s="16" t="n">
         <v>298</v>
       </c>
-      <c r="I19" s="9" t="n">
+      <c r="I19" s="17" t="n">
         <v>254</v>
       </c>
-      <c r="J19" s="10" t="n">
+      <c r="J19" s="18" t="n">
         <v>179</v>
       </c>
-      <c r="K19" s="11" t="n">
+      <c r="K19" s="19" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>2024Q4</t>
         </is>
       </c>
-      <c r="B20" s="12" t="n">
+      <c r="B20" s="20" t="n">
         <v>2024</v>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D20" s="12" t="n">
+      <c r="D20" s="21" t="n">
         <v>35155</v>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E20" s="21" t="n">
         <v>1031</v>
       </c>
-      <c r="F20" s="12" t="n">
+      <c r="F20" s="21" t="n">
         <v>3469</v>
       </c>
-      <c r="G20" s="12" t="n">
+      <c r="G20" s="21" t="n">
         <v>2807</v>
       </c>
-      <c r="H20" s="12" t="n">
+      <c r="H20" s="21" t="n">
         <v>345</v>
       </c>
-      <c r="I20" s="12" t="n">
+      <c r="I20" s="21" t="n">
         <v>268</v>
       </c>
-      <c r="J20" s="12" t="n">
+      <c r="J20" s="21" t="n">
         <v>121</v>
       </c>
-      <c r="K20" s="12" t="n">
+      <c r="K20" s="21" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>2025Q1</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n">
+      <c r="B21" s="11" t="n">
         <v>2025</v>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="5" t="n">
+      <c r="D21" s="12" t="n">
         <v>33387</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" s="13" t="n">
         <v>1103</v>
       </c>
-      <c r="F21" s="6" t="n">
+      <c r="F21" s="14" t="n">
         <v>3530</v>
       </c>
-      <c r="G21" s="7" t="n">
+      <c r="G21" s="15" t="n">
         <v>2746</v>
       </c>
-      <c r="H21" s="8" t="n">
+      <c r="H21" s="16" t="n">
         <v>322</v>
       </c>
-      <c r="I21" s="9" t="n">
+      <c r="I21" s="17" t="n">
         <v>287</v>
       </c>
-      <c r="J21" s="10" t="n">
+      <c r="J21" s="18" t="n">
         <v>256</v>
       </c>
-      <c r="K21" s="11" t="n">
+      <c r="K21" s="19" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>2025Q2</t>
         </is>
       </c>
-      <c r="B22" s="12" t="n">
+      <c r="B22" s="20" t="n">
         <v>2025</v>
       </c>
-      <c r="C22" s="12" t="n">
+      <c r="C22" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D22" s="12" t="n">
+      <c r="D22" s="21" t="n">
         <v>34595</v>
       </c>
-      <c r="E22" s="12" t="n">
+      <c r="E22" s="21" t="n">
         <v>913</v>
       </c>
-      <c r="F22" s="12" t="n">
+      <c r="F22" s="21" t="n">
         <v>2995</v>
       </c>
-      <c r="G22" s="12" t="n">
+      <c r="G22" s="21" t="n">
         <v>2323</v>
       </c>
-      <c r="H22" s="12" t="n">
+      <c r="H22" s="21" t="n">
         <v>346</v>
       </c>
-      <c r="I22" s="12" t="n">
+      <c r="I22" s="21" t="n">
         <v>270</v>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J22" s="21" t="n">
         <v>126</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="K22" s="21" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>2025Q3</t>
         </is>
       </c>
-      <c r="B23" s="4" t="n">
+      <c r="B23" s="11" t="n">
         <v>2025</v>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C23" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="D23" s="5" t="n">
+      <c r="D23" s="12" t="n">
         <v>40612</v>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="13" t="n">
         <v>764</v>
       </c>
-      <c r="F23" s="6" t="n">
+      <c r="F23" s="14" t="n">
         <v>3086</v>
       </c>
-      <c r="G23" s="7" t="n">
+      <c r="G23" s="15" t="n">
         <v>2294</v>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="H23" s="16" t="n">
         <v>433</v>
       </c>
-      <c r="I23" s="9" t="n">
+      <c r="I23" s="17" t="n">
         <v>323</v>
       </c>
-      <c r="J23" s="10" t="n">
+      <c r="J23" s="18" t="n">
         <v>72</v>
       </c>
-      <c r="K23" s="11" t="n">
+      <c r="K23" s="19" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>2025Q4</t>
         </is>
       </c>
-      <c r="B24" s="12" t="n">
+      <c r="B24" s="20" t="n">
         <v>2025</v>
       </c>
-      <c r="C24" s="12" t="n">
+      <c r="C24" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D24" s="12" t="n">
+      <c r="D24" s="21" t="n">
         <v>39393</v>
       </c>
-      <c r="E24" s="12" t="n">
+      <c r="E24" s="21" t="n">
         <v>702</v>
       </c>
-      <c r="F24" s="12" t="n">
+      <c r="F24" s="21" t="n">
         <v>2903</v>
       </c>
-      <c r="G24" s="12" t="n">
+      <c r="G24" s="21" t="n">
         <v>2220</v>
       </c>
-      <c r="H24" s="12" t="n">
+      <c r="H24" s="21" t="n">
         <v>431</v>
       </c>
-      <c r="I24" s="12" t="n">
+      <c r="I24" s="21" t="n">
         <v>252</v>
       </c>
-      <c r="J24" s="12" t="n">
+      <c r="J24" s="21" t="n">
         <v>63</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="K24" s="21" t="n">
         <v>11</v>
       </c>
     </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>2021-2025</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D25" s="23" t="n">
+        <v>606302</v>
+      </c>
+      <c r="E25" s="23" t="n">
+        <v>13038</v>
+      </c>
+      <c r="F25" s="23" t="n">
+        <v>44431</v>
+      </c>
+      <c r="G25" s="23" t="n">
+        <v>31948</v>
+      </c>
+      <c r="H25" s="23" t="n">
+        <v>6523</v>
+      </c>
+      <c r="I25" s="23" t="n">
+        <v>5035</v>
+      </c>
+      <c r="J25" s="23" t="n">
+        <v>1970</v>
+      </c>
+      <c r="K25" s="23" t="n">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1"/>
+    <row r="27" ht="15" customHeight="1"/>
+    <row r="28" ht="15" customHeight="1"/>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>Drug Names by Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Somatropin Only</t>
+        </is>
+      </c>
+      <c r="B30" s="25" t="n"/>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Levothyroxine Only</t>
+        </is>
+      </c>
+      <c r="D30" s="25" t="n"/>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Hydrocortisone Only</t>
+        </is>
+      </c>
+      <c r="F30" s="25" t="n"/>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>Leuprolide Only</t>
+        </is>
+      </c>
+      <c r="H30" s="25" t="n"/>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t>Methimazole Only</t>
+        </is>
+      </c>
+      <c r="J30" s="25" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="26" t="inlineStr">
+        <is>
+          <t>1. GENOTROPIN</t>
+        </is>
+      </c>
+      <c r="B31" s="25" t="n"/>
+      <c r="C31" s="26" t="inlineStr">
+        <is>
+          <t>1. LEVOTHYROXINE</t>
+        </is>
+      </c>
+      <c r="D31" s="25" t="n"/>
+      <c r="E31" s="26" t="inlineStr">
+        <is>
+          <t>1. HYDROCORTISONE</t>
+        </is>
+      </c>
+      <c r="F31" s="25" t="n"/>
+      <c r="G31" s="26" t="inlineStr">
+        <is>
+          <t>1. ELIGARD</t>
+        </is>
+      </c>
+      <c r="H31" s="25" t="n"/>
+      <c r="I31" s="26" t="inlineStr">
+        <is>
+          <t>1. METHIMAZOLE</t>
+        </is>
+      </c>
+      <c r="J31" s="25" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="26" t="inlineStr">
+        <is>
+          <t>2. OMNITROPE</t>
+        </is>
+      </c>
+      <c r="B32" s="25" t="n"/>
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>2. SYNTHROID</t>
+        </is>
+      </c>
+      <c r="D32" s="25" t="n"/>
+      <c r="E32" s="26" t="inlineStr">
+        <is>
+          <t>2. HYDROCORTISONE / LACTATE</t>
+        </is>
+      </c>
+      <c r="F32" s="25" t="n"/>
+      <c r="G32" s="26" t="inlineStr">
+        <is>
+          <t>2. LEUPROLIDE ACETATE</t>
+        </is>
+      </c>
+      <c r="H32" s="25" t="n"/>
+      <c r="I32" s="26" t="inlineStr"/>
+      <c r="J32" s="25" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>3. NORDITROPIN</t>
+        </is>
+      </c>
+      <c r="B33" s="25" t="n"/>
+      <c r="C33" s="26" t="inlineStr">
+        <is>
+          <t>3. LEVOTHYROXINE SODIUM</t>
+        </is>
+      </c>
+      <c r="D33" s="25" t="n"/>
+      <c r="E33" s="26" t="inlineStr"/>
+      <c r="F33" s="25" t="n"/>
+      <c r="G33" s="26" t="inlineStr">
+        <is>
+          <t>3. FENSOLVI</t>
+        </is>
+      </c>
+      <c r="H33" s="25" t="n"/>
+      <c r="I33" s="26" t="inlineStr"/>
+      <c r="J33" s="25" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="26" t="inlineStr">
+        <is>
+          <t>4. SAIZEN</t>
+        </is>
+      </c>
+      <c r="B34" s="25" t="n"/>
+      <c r="C34" s="26" t="inlineStr"/>
+      <c r="D34" s="25" t="n"/>
+      <c r="E34" s="26" t="inlineStr"/>
+      <c r="F34" s="25" t="n"/>
+      <c r="G34" s="26" t="inlineStr">
+        <is>
+          <t>4. SUPPRELIN LA</t>
+        </is>
+      </c>
+      <c r="H34" s="25" t="n"/>
+      <c r="I34" s="26" t="inlineStr"/>
+      <c r="J34" s="25" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="26" t="inlineStr">
+        <is>
+          <t>5. NUTROPIN AQ</t>
+        </is>
+      </c>
+      <c r="B35" s="25" t="n"/>
+      <c r="C35" s="26" t="inlineStr"/>
+      <c r="D35" s="25" t="n"/>
+      <c r="E35" s="26" t="inlineStr"/>
+      <c r="F35" s="25" t="n"/>
+      <c r="G35" s="26" t="inlineStr">
+        <is>
+          <t>5. TRIPTODUR</t>
+        </is>
+      </c>
+      <c r="H35" s="25" t="n"/>
+      <c r="I35" s="26" t="inlineStr"/>
+      <c r="J35" s="25" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="26" t="inlineStr">
+        <is>
+          <t>6. NGENLA</t>
+        </is>
+      </c>
+      <c r="B36" s="25" t="n"/>
+      <c r="C36" s="26" t="inlineStr"/>
+      <c r="D36" s="25" t="n"/>
+      <c r="E36" s="26" t="inlineStr"/>
+      <c r="F36" s="25" t="n"/>
+      <c r="G36" s="26" t="inlineStr"/>
+      <c r="H36" s="25" t="n"/>
+      <c r="I36" s="26" t="inlineStr"/>
+      <c r="J36" s="25" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="26" t="inlineStr">
+        <is>
+          <t>7. SOMATROPIN</t>
+        </is>
+      </c>
+      <c r="B37" s="25" t="n"/>
+      <c r="C37" s="26" t="inlineStr"/>
+      <c r="D37" s="25" t="n"/>
+      <c r="E37" s="26" t="inlineStr"/>
+      <c r="F37" s="25" t="n"/>
+      <c r="G37" s="26" t="inlineStr"/>
+      <c r="H37" s="25" t="n"/>
+      <c r="I37" s="26" t="inlineStr"/>
+      <c r="J37" s="25" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="43">
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="I33:J33"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="A29:K29"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A34:B34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>